<commit_message>
Regenerate FPSO Forte spreadsheet from corrected REV0 file
The corrected file changed the Recusadas sheet's Recusadas total from
US$ 4.943 to US$ 42.818.881,74, and shifted its monthly Service/Material
block by +2 columns (now aligned with "Geral - Em análise" instead of
the previous mismatched-header offset). Re-verified via brute-force
column search (0/99 row mismatches at the new offset) and cross-checked
the Recusadas CAPEX+Contar total against the corrected Overview sheet
figure. "Geral - Em análise" was unaffected (still matches
US$ 137.789.023,16).
</commit_message>
<xml_diff>
--- a/Plano_Integrado_-_FORTE_REV0_enxuta.xlsx
+++ b/Plano_Integrado_-_FORTE_REV0_enxuta.xlsx
@@ -17614,7 +17614,7 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>7</v>
+        <v>63636.36</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
@@ -17643,7 +17643,7 @@
         <v>0</v>
       </c>
       <c r="H2" t="n">
-        <v>7</v>
+        <v>63636.36</v>
       </c>
       <c r="I2" t="n">
         <v>0</v>
@@ -17675,7 +17675,7 @@
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>0</v>
+        <v>90909.09</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
@@ -17704,7 +17704,7 @@
         <v>0</v>
       </c>
       <c r="H3" t="n">
-        <v>0</v>
+        <v>90909.09</v>
       </c>
       <c r="I3" t="n">
         <v>0</v>
@@ -17736,7 +17736,7 @@
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>0</v>
+        <v>2538461.5</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
@@ -17762,19 +17762,19 @@
         <v>0</v>
       </c>
       <c r="G4" t="n">
-        <v>0</v>
+        <v>507692.3</v>
       </c>
       <c r="H4" t="n">
-        <v>0</v>
+        <v>507692.3</v>
       </c>
       <c r="I4" t="n">
-        <v>0</v>
+        <v>507692.3</v>
       </c>
       <c r="J4" t="n">
-        <v>0</v>
+        <v>507692.3</v>
       </c>
       <c r="K4" t="n">
-        <v>0</v>
+        <v>507692.3</v>
       </c>
       <c r="L4" t="n">
         <v>0</v>
@@ -17797,7 +17797,7 @@
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>0</v>
+        <v>6360000</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
@@ -17823,19 +17823,19 @@
         <v>0</v>
       </c>
       <c r="G5" t="n">
-        <v>0</v>
+        <v>1272000</v>
       </c>
       <c r="H5" t="n">
-        <v>0</v>
+        <v>1272000</v>
       </c>
       <c r="I5" t="n">
-        <v>0</v>
+        <v>1272000</v>
       </c>
       <c r="J5" t="n">
-        <v>0</v>
+        <v>1272000</v>
       </c>
       <c r="K5" t="n">
-        <v>0</v>
+        <v>1272000</v>
       </c>
       <c r="L5" t="n">
         <v>0</v>
@@ -17858,7 +17858,7 @@
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>0</v>
+        <v>500000</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
@@ -17908,7 +17908,7 @@
         <v>0</v>
       </c>
       <c r="O6" t="n">
-        <v>0</v>
+        <v>500000</v>
       </c>
       <c r="P6" t="n">
         <v>0</v>
@@ -17919,7 +17919,7 @@
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>139</v>
+        <v>400800</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
@@ -17942,16 +17942,16 @@
         </is>
       </c>
       <c r="F7" t="n">
-        <v>36</v>
+        <v>56000</v>
       </c>
       <c r="G7" t="n">
-        <v>52</v>
+        <v>240000</v>
       </c>
       <c r="H7" t="n">
-        <v>38</v>
+        <v>68800</v>
       </c>
       <c r="I7" t="n">
-        <v>13</v>
+        <v>36000</v>
       </c>
       <c r="J7" t="n">
         <v>0</v>
@@ -17980,7 +17980,7 @@
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
@@ -18030,18 +18030,18 @@
         <v>0</v>
       </c>
       <c r="O8" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="P8" t="n">
         <v>0</v>
       </c>
       <c r="Q8" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>16</v>
+        <v>0</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
@@ -18064,7 +18064,7 @@
         </is>
       </c>
       <c r="F9" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="G9" t="n">
         <v>0</v>
@@ -18073,7 +18073,7 @@
         <v>0</v>
       </c>
       <c r="I9" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="J9" t="n">
         <v>0</v>
@@ -18082,7 +18082,7 @@
         <v>0</v>
       </c>
       <c r="L9" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="M9" t="n">
         <v>0</v>
@@ -18094,7 +18094,7 @@
         <v>0</v>
       </c>
       <c r="P9" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="Q9" t="n">
         <v>0</v>
@@ -18102,7 +18102,7 @@
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>39</v>
+        <v>135519.13</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
@@ -18128,10 +18128,10 @@
         <v>0</v>
       </c>
       <c r="G10" t="n">
-        <v>16</v>
+        <v>135519.13</v>
       </c>
       <c r="H10" t="n">
-        <v>23</v>
+        <v>0</v>
       </c>
       <c r="I10" t="n">
         <v>0</v>
@@ -18163,7 +18163,7 @@
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>42</v>
+        <v>0</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
@@ -18186,7 +18186,7 @@
         </is>
       </c>
       <c r="F11" t="n">
-        <v>42</v>
+        <v>0</v>
       </c>
       <c r="G11" t="n">
         <v>0</v>
@@ -18224,7 +18224,7 @@
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>92</v>
+        <v>0</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
@@ -18247,13 +18247,13 @@
         </is>
       </c>
       <c r="F12" t="n">
-        <v>39</v>
+        <v>0</v>
       </c>
       <c r="G12" t="n">
-        <v>39</v>
+        <v>0</v>
       </c>
       <c r="H12" t="n">
-        <v>14</v>
+        <v>0</v>
       </c>
       <c r="I12" t="n">
         <v>0</v>
@@ -18285,7 +18285,7 @@
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>92</v>
+        <v>0</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
@@ -18308,13 +18308,13 @@
         </is>
       </c>
       <c r="F13" t="n">
-        <v>39</v>
+        <v>0</v>
       </c>
       <c r="G13" t="n">
-        <v>39</v>
+        <v>0</v>
       </c>
       <c r="H13" t="n">
-        <v>14</v>
+        <v>0</v>
       </c>
       <c r="I13" t="n">
         <v>0</v>
@@ -18346,7 +18346,7 @@
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>372</v>
+        <v>0</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
@@ -18369,45 +18369,45 @@
         </is>
       </c>
       <c r="F14" t="n">
-        <v>31</v>
+        <v>0</v>
       </c>
       <c r="G14" t="n">
-        <v>31</v>
+        <v>0</v>
       </c>
       <c r="H14" t="n">
-        <v>31</v>
+        <v>0</v>
       </c>
       <c r="I14" t="n">
-        <v>31</v>
+        <v>0</v>
       </c>
       <c r="J14" t="n">
-        <v>31</v>
+        <v>0</v>
       </c>
       <c r="K14" t="n">
-        <v>31</v>
+        <v>0</v>
       </c>
       <c r="L14" t="n">
-        <v>31</v>
+        <v>0</v>
       </c>
       <c r="M14" t="n">
-        <v>31</v>
+        <v>0</v>
       </c>
       <c r="N14" t="n">
-        <v>31</v>
+        <v>0</v>
       </c>
       <c r="O14" t="n">
-        <v>31</v>
+        <v>0</v>
       </c>
       <c r="P14" t="n">
-        <v>31</v>
+        <v>0</v>
       </c>
       <c r="Q14" t="n">
-        <v>31</v>
+        <v>0</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>12</v>
+        <v>100000</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
@@ -18430,7 +18430,7 @@
         </is>
       </c>
       <c r="F15" t="n">
-        <v>12</v>
+        <v>100000</v>
       </c>
       <c r="G15" t="n">
         <v>0</v>
@@ -18468,7 +18468,7 @@
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>21</v>
+        <v>190000</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
@@ -18497,7 +18497,7 @@
         <v>0</v>
       </c>
       <c r="H16" t="n">
-        <v>21</v>
+        <v>190000</v>
       </c>
       <c r="I16" t="n">
         <v>0</v>
@@ -18529,7 +18529,7 @@
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>20</v>
+        <v>330000</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
@@ -18552,7 +18552,7 @@
         </is>
       </c>
       <c r="F17" t="n">
-        <v>20</v>
+        <v>330000</v>
       </c>
       <c r="G17" t="n">
         <v>0</v>
@@ -18590,7 +18590,7 @@
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>0</v>
+        <v>2000000</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
@@ -18625,25 +18625,25 @@
         <v>0</v>
       </c>
       <c r="J18" t="n">
-        <v>0</v>
+        <v>500000</v>
       </c>
       <c r="K18" t="n">
         <v>0</v>
       </c>
       <c r="L18" t="n">
-        <v>0</v>
+        <v>500000</v>
       </c>
       <c r="M18" t="n">
         <v>0</v>
       </c>
       <c r="N18" t="n">
-        <v>0</v>
+        <v>500000</v>
       </c>
       <c r="O18" t="n">
         <v>0</v>
       </c>
       <c r="P18" t="n">
-        <v>0</v>
+        <v>500000</v>
       </c>
       <c r="Q18" t="n">
         <v>0</v>
@@ -18651,7 +18651,7 @@
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>0</v>
+        <v>772000</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
@@ -18698,7 +18698,7 @@
         <v>0</v>
       </c>
       <c r="N19" t="n">
-        <v>0</v>
+        <v>772000</v>
       </c>
       <c r="O19" t="n">
         <v>0</v>
@@ -18712,7 +18712,7 @@
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>60</v>
+        <v>0.13</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
@@ -18735,45 +18735,45 @@
         </is>
       </c>
       <c r="F20" t="n">
-        <v>5</v>
+        <v>0.02</v>
       </c>
       <c r="G20" t="n">
-        <v>5</v>
+        <v>0.01</v>
       </c>
       <c r="H20" t="n">
-        <v>5</v>
+        <v>0.01</v>
       </c>
       <c r="I20" t="n">
-        <v>5</v>
+        <v>0.01</v>
       </c>
       <c r="J20" t="n">
-        <v>5</v>
+        <v>0.01</v>
       </c>
       <c r="K20" t="n">
-        <v>5</v>
+        <v>0.01</v>
       </c>
       <c r="L20" t="n">
-        <v>5</v>
+        <v>0.01</v>
       </c>
       <c r="M20" t="n">
-        <v>5</v>
+        <v>0.01</v>
       </c>
       <c r="N20" t="n">
-        <v>5</v>
+        <v>0.01</v>
       </c>
       <c r="O20" t="n">
-        <v>5</v>
+        <v>0.01</v>
       </c>
       <c r="P20" t="n">
-        <v>5</v>
+        <v>0.01</v>
       </c>
       <c r="Q20" t="n">
-        <v>5</v>
+        <v>0.01</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>16</v>
+        <v>90000</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
@@ -18820,7 +18820,7 @@
         <v>0</v>
       </c>
       <c r="N21" t="n">
-        <v>16</v>
+        <v>90000</v>
       </c>
       <c r="O21" t="n">
         <v>0</v>
@@ -18834,7 +18834,7 @@
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>0</v>
+        <v>906000</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
@@ -18887,7 +18887,7 @@
         <v>0</v>
       </c>
       <c r="P22" t="n">
-        <v>0</v>
+        <v>906000</v>
       </c>
       <c r="Q22" t="n">
         <v>0</v>
@@ -18895,7 +18895,7 @@
     </row>
     <row r="23">
       <c r="A23" t="n">
-        <v>0</v>
+        <v>10472.72727272727</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
@@ -18924,7 +18924,7 @@
         <v>0</v>
       </c>
       <c r="H23" t="n">
-        <v>0</v>
+        <v>10472.72727272727</v>
       </c>
       <c r="I23" t="n">
         <v>0</v>
@@ -18956,7 +18956,7 @@
     </row>
     <row r="24">
       <c r="A24" t="n">
-        <v>51</v>
+        <v>3243855.32</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
@@ -18991,7 +18991,7 @@
         <v>0</v>
       </c>
       <c r="J24" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="K24" t="n">
         <v>0</v>
@@ -19009,15 +19009,15 @@
         <v>0</v>
       </c>
       <c r="P24" t="n">
-        <v>34</v>
+        <v>720856.74</v>
       </c>
       <c r="Q24" t="n">
-        <v>10</v>
+        <v>2522998.58</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>17</v>
+        <v>164000</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
@@ -19058,7 +19058,7 @@
         <v>0</v>
       </c>
       <c r="L25" t="n">
-        <v>17</v>
+        <v>164000</v>
       </c>
       <c r="M25" t="n">
         <v>0</v>
@@ -19078,7 +19078,7 @@
     </row>
     <row r="26">
       <c r="A26" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="B26" t="inlineStr">
         <is>
@@ -19101,7 +19101,7 @@
         </is>
       </c>
       <c r="F26" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="G26" t="n">
         <v>0</v>
@@ -19139,7 +19139,7 @@
     </row>
     <row r="27">
       <c r="A27" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="B27" t="inlineStr">
         <is>
@@ -19171,7 +19171,7 @@
         <v>0</v>
       </c>
       <c r="I27" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="J27" t="n">
         <v>0</v>
@@ -19200,7 +19200,7 @@
     </row>
     <row r="28">
       <c r="A28" t="n">
-        <v>100</v>
+        <v>838310</v>
       </c>
       <c r="B28" t="inlineStr">
         <is>
@@ -19223,7 +19223,7 @@
         </is>
       </c>
       <c r="F28" t="n">
-        <v>0</v>
+        <v>74545</v>
       </c>
       <c r="G28" t="n">
         <v>0</v>
@@ -19247,13 +19247,13 @@
         <v>0</v>
       </c>
       <c r="N28" t="n">
-        <v>33</v>
+        <v>677037</v>
       </c>
       <c r="O28" t="n">
-        <v>34</v>
+        <v>43364</v>
       </c>
       <c r="P28" t="n">
-        <v>33</v>
+        <v>43364</v>
       </c>
       <c r="Q28" t="n">
         <v>0</v>
@@ -19261,7 +19261,7 @@
     </row>
     <row r="29">
       <c r="A29" t="n">
-        <v>130</v>
+        <v>1427496</v>
       </c>
       <c r="B29" t="inlineStr">
         <is>
@@ -19287,7 +19287,7 @@
         <v>0</v>
       </c>
       <c r="G29" t="n">
-        <v>0</v>
+        <v>74545</v>
       </c>
       <c r="H29" t="n">
         <v>0</v>
@@ -19308,21 +19308,21 @@
         <v>0</v>
       </c>
       <c r="N29" t="n">
-        <v>37</v>
+        <v>1070134</v>
       </c>
       <c r="O29" t="n">
-        <v>38</v>
+        <v>128818</v>
       </c>
       <c r="P29" t="n">
-        <v>37</v>
+        <v>128818</v>
       </c>
       <c r="Q29" t="n">
-        <v>18</v>
+        <v>25181</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
-        <v>18</v>
+        <v>160000</v>
       </c>
       <c r="B30" t="inlineStr">
         <is>
@@ -19348,7 +19348,7 @@
         <v>0</v>
       </c>
       <c r="G30" t="n">
-        <v>18</v>
+        <v>160000</v>
       </c>
       <c r="H30" t="n">
         <v>0</v>
@@ -19383,7 +19383,7 @@
     </row>
     <row r="31">
       <c r="A31" t="n">
-        <v>61</v>
+        <v>620072.72</v>
       </c>
       <c r="B31" t="inlineStr">
         <is>
@@ -19427,10 +19427,10 @@
         <v>0</v>
       </c>
       <c r="M31" t="n">
-        <v>33</v>
+        <v>310036.36</v>
       </c>
       <c r="N31" t="n">
-        <v>28</v>
+        <v>310036.36</v>
       </c>
       <c r="O31" t="n">
         <v>0</v>
@@ -19444,7 +19444,7 @@
     </row>
     <row r="32">
       <c r="A32" t="n">
-        <v>4</v>
+        <v>100000</v>
       </c>
       <c r="B32" t="inlineStr">
         <is>
@@ -19479,7 +19479,7 @@
         <v>0</v>
       </c>
       <c r="J32" t="n">
-        <v>4</v>
+        <v>100000</v>
       </c>
       <c r="K32" t="n">
         <v>0</v>
@@ -19505,7 +19505,7 @@
     </row>
     <row r="33">
       <c r="A33" t="n">
-        <v>51</v>
+        <v>81000</v>
       </c>
       <c r="B33" t="inlineStr">
         <is>
@@ -19531,10 +19531,10 @@
         <v>0</v>
       </c>
       <c r="G33" t="n">
-        <v>18</v>
+        <v>27000</v>
       </c>
       <c r="H33" t="n">
-        <v>33</v>
+        <v>54000</v>
       </c>
       <c r="I33" t="n">
         <v>0</v>
@@ -19566,7 +19566,7 @@
     </row>
     <row r="34">
       <c r="A34" t="n">
-        <v>43</v>
+        <v>40000</v>
       </c>
       <c r="B34" t="inlineStr">
         <is>
@@ -19589,7 +19589,7 @@
         </is>
       </c>
       <c r="F34" t="n">
-        <v>16</v>
+        <v>10000</v>
       </c>
       <c r="G34" t="n">
         <v>0</v>
@@ -19598,7 +19598,7 @@
         <v>0</v>
       </c>
       <c r="I34" t="n">
-        <v>9</v>
+        <v>10000</v>
       </c>
       <c r="J34" t="n">
         <v>0</v>
@@ -19607,7 +19607,7 @@
         <v>0</v>
       </c>
       <c r="L34" t="n">
-        <v>9</v>
+        <v>10000</v>
       </c>
       <c r="M34" t="n">
         <v>0</v>
@@ -19616,7 +19616,7 @@
         <v>0</v>
       </c>
       <c r="O34" t="n">
-        <v>9</v>
+        <v>10000</v>
       </c>
       <c r="P34" t="n">
         <v>0</v>
@@ -19627,7 +19627,7 @@
     </row>
     <row r="35">
       <c r="A35" t="n">
-        <v>8</v>
+        <v>10000</v>
       </c>
       <c r="B35" t="inlineStr">
         <is>
@@ -19653,7 +19653,7 @@
         <v>0</v>
       </c>
       <c r="G35" t="n">
-        <v>8</v>
+        <v>10000</v>
       </c>
       <c r="H35" t="n">
         <v>0</v>
@@ -19688,7 +19688,7 @@
     </row>
     <row r="36">
       <c r="A36" t="n">
-        <v>12</v>
+        <v>5000</v>
       </c>
       <c r="B36" t="inlineStr">
         <is>
@@ -19735,7 +19735,7 @@
         <v>0</v>
       </c>
       <c r="N36" t="n">
-        <v>12</v>
+        <v>5000</v>
       </c>
       <c r="O36" t="n">
         <v>0</v>
@@ -19749,7 +19749,7 @@
     </row>
     <row r="37">
       <c r="A37" t="n">
-        <v>475</v>
+        <v>1955045.545454546</v>
       </c>
       <c r="B37" t="inlineStr">
         <is>
@@ -19778,22 +19778,22 @@
         <v>0</v>
       </c>
       <c r="H37" t="n">
-        <v>88</v>
+        <v>384381.8181818182</v>
       </c>
       <c r="I37" t="n">
-        <v>88</v>
+        <v>384381.8181818182</v>
       </c>
       <c r="J37" t="n">
-        <v>56</v>
+        <v>172309.0909090909</v>
       </c>
       <c r="K37" t="n">
-        <v>81</v>
+        <v>337990.9090909091</v>
       </c>
       <c r="L37" t="n">
-        <v>81</v>
+        <v>337990.9090909091</v>
       </c>
       <c r="M37" t="n">
-        <v>81</v>
+        <v>337991</v>
       </c>
       <c r="N37" t="n">
         <v>0</v>
@@ -19810,7 +19810,7 @@
     </row>
     <row r="38">
       <c r="A38" t="n">
-        <v>448</v>
+        <v>2140174.636363636</v>
       </c>
       <c r="B38" t="inlineStr">
         <is>
@@ -19839,22 +19839,22 @@
         <v>0</v>
       </c>
       <c r="H38" t="n">
-        <v>45</v>
+        <v>119785.9090909091</v>
       </c>
       <c r="I38" t="n">
-        <v>73</v>
+        <v>343386.2727272727</v>
       </c>
       <c r="J38" t="n">
-        <v>180</v>
+        <v>1197859.090909091</v>
       </c>
       <c r="K38" t="n">
-        <v>70</v>
+        <v>319429.0909090909</v>
       </c>
       <c r="L38" t="n">
-        <v>40</v>
+        <v>79857.27272727272</v>
       </c>
       <c r="M38" t="n">
-        <v>40</v>
+        <v>79857</v>
       </c>
       <c r="N38" t="n">
         <v>0</v>
@@ -19871,7 +19871,7 @@
     </row>
     <row r="39">
       <c r="A39" t="n">
-        <v>270</v>
+        <v>1193891.363636364</v>
       </c>
       <c r="B39" t="inlineStr">
         <is>
@@ -19900,22 +19900,22 @@
         <v>0</v>
       </c>
       <c r="H39" t="n">
-        <v>40</v>
+        <v>132654.5454545454</v>
       </c>
       <c r="I39" t="n">
-        <v>40</v>
+        <v>132654.5454545454</v>
       </c>
       <c r="J39" t="n">
-        <v>70</v>
+        <v>530618.1818181818</v>
       </c>
       <c r="K39" t="n">
-        <v>40</v>
+        <v>132654.5454545454</v>
       </c>
       <c r="L39" t="n">
-        <v>40</v>
+        <v>132654.5454545454</v>
       </c>
       <c r="M39" t="n">
-        <v>40</v>
+        <v>132655</v>
       </c>
       <c r="N39" t="n">
         <v>0</v>
@@ -19932,7 +19932,7 @@
     </row>
     <row r="40">
       <c r="A40" t="n">
-        <v>221</v>
+        <v>1191886.527272727</v>
       </c>
       <c r="B40" t="inlineStr">
         <is>
@@ -19967,16 +19967,16 @@
         <v>0</v>
       </c>
       <c r="J40" t="n">
-        <v>44</v>
+        <v>165211.9636363636</v>
       </c>
       <c r="K40" t="n">
-        <v>59</v>
+        <v>342224.7818181818</v>
       </c>
       <c r="L40" t="n">
-        <v>59</v>
+        <v>342224.7818181818</v>
       </c>
       <c r="M40" t="n">
-        <v>59</v>
+        <v>342225</v>
       </c>
       <c r="N40" t="n">
         <v>0</v>
@@ -19993,7 +19993,7 @@
     </row>
     <row r="41">
       <c r="A41" t="n">
-        <v>16</v>
+        <v>383194.8</v>
       </c>
       <c r="B41" t="inlineStr">
         <is>
@@ -20046,7 +20046,7 @@
         <v>0</v>
       </c>
       <c r="P41" t="n">
-        <v>16</v>
+        <v>383194.8</v>
       </c>
       <c r="Q41" t="n">
         <v>0</v>
@@ -20054,7 +20054,7 @@
     </row>
     <row r="42">
       <c r="A42" t="n">
-        <v>16</v>
+        <v>108000</v>
       </c>
       <c r="B42" t="inlineStr">
         <is>
@@ -20092,7 +20092,7 @@
         <v>0</v>
       </c>
       <c r="K42" t="n">
-        <v>16</v>
+        <v>108000</v>
       </c>
       <c r="L42" t="n">
         <v>0</v>
@@ -20115,7 +20115,7 @@
     </row>
     <row r="43">
       <c r="A43" t="n">
-        <v>28</v>
+        <v>2802319.16</v>
       </c>
       <c r="B43" t="inlineStr">
         <is>
@@ -20153,7 +20153,7 @@
         <v>0</v>
       </c>
       <c r="K43" t="n">
-        <v>28</v>
+        <v>2802319.16</v>
       </c>
       <c r="L43" t="n">
         <v>0</v>
@@ -20176,7 +20176,7 @@
     </row>
     <row r="44">
       <c r="A44" t="n">
-        <v>62</v>
+        <v>35312.72727272727</v>
       </c>
       <c r="B44" t="inlineStr">
         <is>
@@ -20199,10 +20199,10 @@
         </is>
       </c>
       <c r="F44" t="n">
-        <v>31</v>
+        <v>17656.36363636364</v>
       </c>
       <c r="G44" t="n">
-        <v>31</v>
+        <v>17656.36363636364</v>
       </c>
       <c r="H44" t="n">
         <v>0</v>
@@ -20237,7 +20237,7 @@
     </row>
     <row r="45">
       <c r="A45" t="n">
-        <v>63</v>
+        <v>375000</v>
       </c>
       <c r="B45" t="inlineStr">
         <is>
@@ -20266,13 +20266,13 @@
         <v>0</v>
       </c>
       <c r="H45" t="n">
-        <v>21</v>
+        <v>125000</v>
       </c>
       <c r="I45" t="n">
         <v>0</v>
       </c>
       <c r="J45" t="n">
-        <v>21</v>
+        <v>125000</v>
       </c>
       <c r="K45" t="n">
         <v>0</v>
@@ -20281,7 +20281,7 @@
         <v>0</v>
       </c>
       <c r="M45" t="n">
-        <v>21</v>
+        <v>125000</v>
       </c>
       <c r="N45" t="n">
         <v>0</v>
@@ -20298,7 +20298,7 @@
     </row>
     <row r="46">
       <c r="A46" t="n">
-        <v>162</v>
+        <v>675981.8181818182</v>
       </c>
       <c r="B46" t="inlineStr">
         <is>
@@ -20336,10 +20336,10 @@
         <v>0</v>
       </c>
       <c r="K46" t="n">
-        <v>81</v>
+        <v>337990.9090909091</v>
       </c>
       <c r="L46" t="n">
-        <v>81</v>
+        <v>337990.9090909091</v>
       </c>
       <c r="M46" t="n">
         <v>0</v>
@@ -20359,7 +20359,7 @@
     </row>
     <row r="47">
       <c r="A47" t="n">
-        <v>110</v>
+        <v>399286.3636363636</v>
       </c>
       <c r="B47" t="inlineStr">
         <is>
@@ -20397,10 +20397,10 @@
         <v>0</v>
       </c>
       <c r="K47" t="n">
-        <v>70</v>
+        <v>319429.0909090909</v>
       </c>
       <c r="L47" t="n">
-        <v>40</v>
+        <v>79857.27272727272</v>
       </c>
       <c r="M47" t="n">
         <v>0</v>
@@ -20420,7 +20420,7 @@
     </row>
     <row r="48">
       <c r="A48" t="n">
-        <v>69</v>
+        <v>238090.9090909091</v>
       </c>
       <c r="B48" t="inlineStr">
         <is>
@@ -20458,10 +20458,10 @@
         <v>0</v>
       </c>
       <c r="K48" t="n">
-        <v>36</v>
+        <v>158727.2727272727</v>
       </c>
       <c r="L48" t="n">
-        <v>33</v>
+        <v>79363.63636363637</v>
       </c>
       <c r="M48" t="n">
         <v>0</v>
@@ -20481,7 +20481,7 @@
     </row>
     <row r="49">
       <c r="A49" t="n">
-        <v>80</v>
+        <v>265309.0909090909</v>
       </c>
       <c r="B49" t="inlineStr">
         <is>
@@ -20519,10 +20519,10 @@
         <v>0</v>
       </c>
       <c r="K49" t="n">
-        <v>40</v>
+        <v>132654.5454545454</v>
       </c>
       <c r="L49" t="n">
-        <v>40</v>
+        <v>132654.5454545454</v>
       </c>
       <c r="M49" t="n">
         <v>0</v>
@@ -20542,7 +20542,7 @@
     </row>
     <row r="50">
       <c r="A50" t="n">
-        <v>35</v>
+        <v>66327.27272727272</v>
       </c>
       <c r="B50" t="inlineStr">
         <is>
@@ -20580,7 +20580,7 @@
         <v>0</v>
       </c>
       <c r="K50" t="n">
-        <v>35</v>
+        <v>66327.27272727272</v>
       </c>
       <c r="L50" t="n">
         <v>0</v>
@@ -20603,7 +20603,7 @@
     </row>
     <row r="51">
       <c r="A51" t="n">
-        <v>118</v>
+        <v>684449.5636363636</v>
       </c>
       <c r="B51" t="inlineStr">
         <is>
@@ -20641,10 +20641,10 @@
         <v>0</v>
       </c>
       <c r="K51" t="n">
-        <v>59</v>
+        <v>342224.7818181818</v>
       </c>
       <c r="L51" t="n">
-        <v>59</v>
+        <v>342224.7818181818</v>
       </c>
       <c r="M51" t="n">
         <v>0</v>
@@ -20664,7 +20664,7 @@
     </row>
     <row r="52">
       <c r="A52" t="n">
-        <v>176</v>
+        <v>768763.64</v>
       </c>
       <c r="B52" t="inlineStr">
         <is>
@@ -20693,10 +20693,10 @@
         <v>0</v>
       </c>
       <c r="H52" t="n">
-        <v>88</v>
+        <v>384381.82</v>
       </c>
       <c r="I52" t="n">
-        <v>88</v>
+        <v>384381.82</v>
       </c>
       <c r="J52" t="n">
         <v>0</v>
@@ -20725,7 +20725,7 @@
     </row>
     <row r="53">
       <c r="A53" t="n">
-        <v>118</v>
+        <v>463172.1827272727</v>
       </c>
       <c r="B53" t="inlineStr">
         <is>
@@ -20754,10 +20754,10 @@
         <v>0</v>
       </c>
       <c r="H53" t="n">
-        <v>45</v>
+        <v>119785.91</v>
       </c>
       <c r="I53" t="n">
-        <v>73</v>
+        <v>343386.2727272727</v>
       </c>
       <c r="J53" t="n">
         <v>0</v>
@@ -20786,7 +20786,7 @@
     </row>
     <row r="54">
       <c r="A54" t="n">
-        <v>68</v>
+        <v>211636.36</v>
       </c>
       <c r="B54" t="inlineStr">
         <is>
@@ -20815,10 +20815,10 @@
         <v>0</v>
       </c>
       <c r="H54" t="n">
-        <v>34</v>
+        <v>105818.18</v>
       </c>
       <c r="I54" t="n">
-        <v>34</v>
+        <v>105818.18</v>
       </c>
       <c r="J54" t="n">
         <v>0</v>
@@ -20847,7 +20847,7 @@
     </row>
     <row r="55">
       <c r="A55" t="n">
-        <v>122</v>
+        <v>371247.1</v>
       </c>
       <c r="B55" t="inlineStr">
         <is>
@@ -20870,16 +20870,16 @@
         </is>
       </c>
       <c r="F55" t="n">
-        <v>21</v>
+        <v>52969</v>
       </c>
       <c r="G55" t="n">
-        <v>21</v>
+        <v>52969</v>
       </c>
       <c r="H55" t="n">
-        <v>40</v>
+        <v>132654.55</v>
       </c>
       <c r="I55" t="n">
-        <v>40</v>
+        <v>132654.55</v>
       </c>
       <c r="J55" t="n">
         <v>0</v>
@@ -20908,7 +20908,7 @@
     </row>
     <row r="56">
       <c r="A56" t="n">
-        <v>108</v>
+        <v>247560.01</v>
       </c>
       <c r="B56" t="inlineStr">
         <is>
@@ -20931,16 +20931,16 @@
         </is>
       </c>
       <c r="F56" t="n">
-        <v>32</v>
+        <v>35312.73</v>
       </c>
       <c r="G56" t="n">
         <v>0</v>
       </c>
       <c r="H56" t="n">
-        <v>38</v>
+        <v>106123.64</v>
       </c>
       <c r="I56" t="n">
-        <v>38</v>
+        <v>106123.64</v>
       </c>
       <c r="J56" t="n">
         <v>0</v>
@@ -20969,7 +20969,7 @@
     </row>
     <row r="57">
       <c r="A57" t="n">
-        <v>6</v>
+        <v>135000</v>
       </c>
       <c r="B57" t="inlineStr">
         <is>
@@ -20995,7 +20995,7 @@
         <v>0</v>
       </c>
       <c r="G57" t="n">
-        <v>6</v>
+        <v>135000</v>
       </c>
       <c r="H57" t="n">
         <v>0</v>
@@ -21030,7 +21030,7 @@
     </row>
     <row r="58">
       <c r="A58" t="n">
-        <v>18</v>
+        <v>600000</v>
       </c>
       <c r="B58" t="inlineStr">
         <is>
@@ -21083,7 +21083,7 @@
         <v>0</v>
       </c>
       <c r="P58" t="n">
-        <v>18</v>
+        <v>600000</v>
       </c>
       <c r="Q58" t="n">
         <v>0</v>
@@ -21091,7 +21091,7 @@
     </row>
     <row r="59">
       <c r="A59" t="n">
-        <v>9</v>
+        <v>90000</v>
       </c>
       <c r="B59" t="inlineStr">
         <is>
@@ -21141,7 +21141,7 @@
         <v>0</v>
       </c>
       <c r="O59" t="n">
-        <v>9</v>
+        <v>90000</v>
       </c>
       <c r="P59" t="n">
         <v>0</v>
@@ -21152,7 +21152,7 @@
     </row>
     <row r="60">
       <c r="A60" t="n">
-        <v>42</v>
+        <v>500000</v>
       </c>
       <c r="B60" t="inlineStr">
         <is>
@@ -21175,13 +21175,13 @@
         </is>
       </c>
       <c r="F60" t="n">
-        <v>21</v>
+        <v>250000</v>
       </c>
       <c r="G60" t="n">
         <v>0</v>
       </c>
       <c r="H60" t="n">
-        <v>21</v>
+        <v>250000</v>
       </c>
       <c r="I60" t="n">
         <v>0</v>
@@ -21213,7 +21213,7 @@
     </row>
     <row r="61">
       <c r="A61" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="B61" t="inlineStr">
         <is>
@@ -21242,7 +21242,7 @@
         <v>0</v>
       </c>
       <c r="H61" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="I61" t="n">
         <v>0</v>
@@ -21274,7 +21274,7 @@
     </row>
     <row r="62">
       <c r="A62" t="n">
-        <v>17</v>
+        <v>120000</v>
       </c>
       <c r="B62" t="inlineStr">
         <is>
@@ -21303,7 +21303,7 @@
         <v>0</v>
       </c>
       <c r="H62" t="n">
-        <v>17</v>
+        <v>120000</v>
       </c>
       <c r="I62" t="n">
         <v>0</v>
@@ -21335,7 +21335,7 @@
     </row>
     <row r="63">
       <c r="A63" t="n">
-        <v>22</v>
+        <v>220000</v>
       </c>
       <c r="B63" t="inlineStr">
         <is>
@@ -21358,7 +21358,7 @@
         </is>
       </c>
       <c r="F63" t="n">
-        <v>22</v>
+        <v>220000</v>
       </c>
       <c r="G63" t="n">
         <v>0</v>
@@ -21396,7 +21396,7 @@
     </row>
     <row r="64">
       <c r="A64" t="n">
-        <v>19</v>
+        <v>170000</v>
       </c>
       <c r="B64" t="inlineStr">
         <is>
@@ -21422,7 +21422,7 @@
         <v>0</v>
       </c>
       <c r="G64" t="n">
-        <v>19</v>
+        <v>170000</v>
       </c>
       <c r="H64" t="n">
         <v>0</v>
@@ -21457,7 +21457,7 @@
     </row>
     <row r="65">
       <c r="A65" t="n">
-        <v>28</v>
+        <v>0</v>
       </c>
       <c r="B65" t="inlineStr">
         <is>
@@ -21483,7 +21483,7 @@
         <v>0</v>
       </c>
       <c r="G65" t="n">
-        <v>28</v>
+        <v>0</v>
       </c>
       <c r="H65" t="n">
         <v>0</v>
@@ -21518,7 +21518,7 @@
     </row>
     <row r="66">
       <c r="A66" t="n">
-        <v>19</v>
+        <v>0</v>
       </c>
       <c r="B66" t="inlineStr">
         <is>
@@ -21544,7 +21544,7 @@
         <v>0</v>
       </c>
       <c r="G66" t="n">
-        <v>19</v>
+        <v>0</v>
       </c>
       <c r="H66" t="n">
         <v>0</v>
@@ -21579,7 +21579,7 @@
     </row>
     <row r="67">
       <c r="A67" t="n">
-        <v>16</v>
+        <v>1050000</v>
       </c>
       <c r="B67" t="inlineStr">
         <is>
@@ -21635,12 +21635,12 @@
         <v>0</v>
       </c>
       <c r="Q67" t="n">
-        <v>16</v>
+        <v>1050000</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="n">
-        <v>21</v>
+        <v>2707401.28</v>
       </c>
       <c r="B68" t="inlineStr">
         <is>
@@ -21675,7 +21675,7 @@
         <v>0</v>
       </c>
       <c r="J68" t="n">
-        <v>21</v>
+        <v>2707401.28</v>
       </c>
       <c r="K68" t="n">
         <v>0</v>
@@ -21701,7 +21701,7 @@
     </row>
     <row r="69">
       <c r="A69" t="n">
-        <v>16</v>
+        <v>63341.2</v>
       </c>
       <c r="B69" t="inlineStr">
         <is>
@@ -21724,7 +21724,7 @@
         </is>
       </c>
       <c r="F69" t="n">
-        <v>16</v>
+        <v>63341.2</v>
       </c>
       <c r="G69" t="n">
         <v>0</v>
@@ -21762,7 +21762,7 @@
     </row>
     <row r="70">
       <c r="A70" t="n">
-        <v>14</v>
+        <v>45506.78</v>
       </c>
       <c r="B70" t="inlineStr">
         <is>
@@ -21785,7 +21785,7 @@
         </is>
       </c>
       <c r="F70" t="n">
-        <v>14</v>
+        <v>45506.78</v>
       </c>
       <c r="G70" t="n">
         <v>0</v>
@@ -21823,7 +21823,7 @@
     </row>
     <row r="71">
       <c r="A71" t="n">
-        <v>17</v>
+        <v>73527.3</v>
       </c>
       <c r="B71" t="inlineStr">
         <is>
@@ -21846,7 +21846,7 @@
         </is>
       </c>
       <c r="F71" t="n">
-        <v>17</v>
+        <v>73527.3</v>
       </c>
       <c r="G71" t="n">
         <v>0</v>
@@ -21884,7 +21884,7 @@
     </row>
     <row r="72">
       <c r="A72" t="n">
-        <v>19</v>
+        <v>326137.26</v>
       </c>
       <c r="B72" t="inlineStr">
         <is>
@@ -21919,7 +21919,7 @@
         <v>0</v>
       </c>
       <c r="J72" t="n">
-        <v>19</v>
+        <v>326137.26</v>
       </c>
       <c r="K72" t="n">
         <v>0</v>
@@ -21945,7 +21945,7 @@
     </row>
     <row r="73">
       <c r="A73" t="n">
-        <v>95</v>
+        <v>873582.52</v>
       </c>
       <c r="B73" t="inlineStr">
         <is>
@@ -21971,16 +21971,16 @@
         <v>0</v>
       </c>
       <c r="G73" t="n">
-        <v>17</v>
+        <v>93712.42</v>
       </c>
       <c r="H73" t="n">
-        <v>17</v>
+        <v>88712.42</v>
       </c>
       <c r="I73" t="n">
-        <v>34</v>
+        <v>481290.43</v>
       </c>
       <c r="J73" t="n">
-        <v>27</v>
+        <v>209867.25</v>
       </c>
       <c r="K73" t="n">
         <v>0</v>
@@ -22006,7 +22006,7 @@
     </row>
     <row r="74">
       <c r="A74" t="n">
-        <v>25</v>
+        <v>127751.44</v>
       </c>
       <c r="B74" t="inlineStr">
         <is>
@@ -22029,7 +22029,7 @@
         </is>
       </c>
       <c r="F74" t="n">
-        <v>25</v>
+        <v>127751.44</v>
       </c>
       <c r="G74" t="n">
         <v>0</v>
@@ -22067,7 +22067,7 @@
     </row>
     <row r="75">
       <c r="A75" t="n">
-        <v>26</v>
+        <v>601818.1800000001</v>
       </c>
       <c r="B75" t="inlineStr">
         <is>
@@ -22099,7 +22099,7 @@
         <v>0</v>
       </c>
       <c r="I75" t="n">
-        <v>26</v>
+        <v>601818.1800000001</v>
       </c>
       <c r="J75" t="n">
         <v>0</v>
@@ -22128,7 +22128,7 @@
     </row>
     <row r="76">
       <c r="A76" t="n">
-        <v>67</v>
+        <v>163424.94</v>
       </c>
       <c r="B76" t="inlineStr">
         <is>
@@ -22151,7 +22151,7 @@
         </is>
       </c>
       <c r="F76" t="n">
-        <v>27</v>
+        <v>80883.42</v>
       </c>
       <c r="G76" t="n">
         <v>0</v>
@@ -22160,10 +22160,10 @@
         <v>0</v>
       </c>
       <c r="I76" t="n">
-        <v>20</v>
+        <v>33770.76</v>
       </c>
       <c r="J76" t="n">
-        <v>20</v>
+        <v>48770.76</v>
       </c>
       <c r="K76" t="n">
         <v>0</v>
@@ -22189,7 +22189,7 @@
     </row>
     <row r="77">
       <c r="A77" t="n">
-        <v>26</v>
+        <v>401589.15</v>
       </c>
       <c r="B77" t="inlineStr">
         <is>
@@ -22212,7 +22212,7 @@
         </is>
       </c>
       <c r="F77" t="n">
-        <v>26</v>
+        <v>401589.15</v>
       </c>
       <c r="G77" t="n">
         <v>0</v>
@@ -22250,7 +22250,7 @@
     </row>
     <row r="78">
       <c r="A78" t="n">
-        <v>20</v>
+        <v>219784.68</v>
       </c>
       <c r="B78" t="inlineStr">
         <is>
@@ -22273,7 +22273,7 @@
         </is>
       </c>
       <c r="F78" t="n">
-        <v>20</v>
+        <v>219784.68</v>
       </c>
       <c r="G78" t="n">
         <v>0</v>
@@ -22311,7 +22311,7 @@
     </row>
     <row r="79">
       <c r="A79" t="n">
-        <v>39</v>
+        <v>164608.88</v>
       </c>
       <c r="B79" t="inlineStr">
         <is>
@@ -22334,10 +22334,10 @@
         </is>
       </c>
       <c r="F79" t="n">
-        <v>20</v>
+        <v>152011.98</v>
       </c>
       <c r="G79" t="n">
-        <v>19</v>
+        <v>12596.9</v>
       </c>
       <c r="H79" t="n">
         <v>0</v>
@@ -22372,7 +22372,7 @@
     </row>
     <row r="80">
       <c r="A80" t="n">
-        <v>16</v>
+        <v>112421.22</v>
       </c>
       <c r="B80" t="inlineStr">
         <is>
@@ -22404,7 +22404,7 @@
         <v>0</v>
       </c>
       <c r="I80" t="n">
-        <v>16</v>
+        <v>112421.22</v>
       </c>
       <c r="J80" t="n">
         <v>0</v>
@@ -22433,7 +22433,7 @@
     </row>
     <row r="81">
       <c r="A81" t="n">
-        <v>28</v>
+        <v>2802317.15</v>
       </c>
       <c r="B81" t="inlineStr">
         <is>
@@ -22468,7 +22468,7 @@
         <v>0</v>
       </c>
       <c r="J81" t="n">
-        <v>28</v>
+        <v>2802317.15</v>
       </c>
       <c r="K81" t="n">
         <v>0</v>
@@ -22494,7 +22494,7 @@
     </row>
     <row r="82">
       <c r="A82" t="n">
-        <v>19</v>
+        <v>154520.7</v>
       </c>
       <c r="B82" t="inlineStr">
         <is>
@@ -22517,7 +22517,7 @@
         </is>
       </c>
       <c r="F82" t="n">
-        <v>19</v>
+        <v>154520.7</v>
       </c>
       <c r="G82" t="n">
         <v>0</v>
@@ -22555,7 +22555,7 @@
     </row>
     <row r="83">
       <c r="A83" t="n">
-        <v>62</v>
+        <v>146000</v>
       </c>
       <c r="B83" t="inlineStr">
         <is>
@@ -22590,7 +22590,7 @@
         <v>0</v>
       </c>
       <c r="J83" t="n">
-        <v>31</v>
+        <v>73000</v>
       </c>
       <c r="K83" t="n">
         <v>0</v>
@@ -22602,7 +22602,7 @@
         <v>0</v>
       </c>
       <c r="N83" t="n">
-        <v>31</v>
+        <v>73000</v>
       </c>
       <c r="O83" t="n">
         <v>0</v>
@@ -22616,7 +22616,7 @@
     </row>
     <row r="84">
       <c r="A84" t="n">
-        <v>104</v>
+        <v>1951344.36</v>
       </c>
       <c r="B84" t="inlineStr">
         <is>
@@ -22666,18 +22666,18 @@
         <v>0</v>
       </c>
       <c r="O84" t="n">
-        <v>39</v>
+        <v>650448.12</v>
       </c>
       <c r="P84" t="n">
-        <v>38</v>
+        <v>650448.12</v>
       </c>
       <c r="Q84" t="n">
-        <v>27</v>
+        <v>650448.12</v>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="n">
-        <v>22</v>
+        <v>340000</v>
       </c>
       <c r="B85" t="inlineStr">
         <is>
@@ -22706,7 +22706,7 @@
         <v>0</v>
       </c>
       <c r="H85" t="n">
-        <v>22</v>
+        <v>340000</v>
       </c>
       <c r="I85" t="n">
         <v>0</v>
@@ -22738,7 +22738,7 @@
     </row>
     <row r="86">
       <c r="A86" t="n">
-        <v>32</v>
+        <v>1400000</v>
       </c>
       <c r="B86" t="inlineStr">
         <is>
@@ -22776,7 +22776,7 @@
         <v>0</v>
       </c>
       <c r="K86" t="n">
-        <v>32</v>
+        <v>1400000</v>
       </c>
       <c r="L86" t="n">
         <v>0</v>
@@ -22799,7 +22799,7 @@
     </row>
     <row r="87">
       <c r="A87" t="n">
-        <v>56</v>
+        <v>172309.0909090909</v>
       </c>
       <c r="B87" t="inlineStr">
         <is>
@@ -22834,7 +22834,7 @@
         <v>0</v>
       </c>
       <c r="J87" t="n">
-        <v>56</v>
+        <v>172309.0909090909</v>
       </c>
       <c r="K87" t="n">
         <v>0</v>
@@ -22860,7 +22860,7 @@
     </row>
     <row r="88">
       <c r="A88" t="n">
-        <v>180</v>
+        <v>1197859.090909091</v>
       </c>
       <c r="B88" t="inlineStr">
         <is>
@@ -22895,7 +22895,7 @@
         <v>0</v>
       </c>
       <c r="J88" t="n">
-        <v>180</v>
+        <v>1197859.090909091</v>
       </c>
       <c r="K88" t="n">
         <v>0</v>
@@ -22921,7 +22921,7 @@
     </row>
     <row r="89">
       <c r="A89" t="n">
-        <v>40</v>
+        <v>264545.4545454545</v>
       </c>
       <c r="B89" t="inlineStr">
         <is>
@@ -22956,7 +22956,7 @@
         <v>0</v>
       </c>
       <c r="J89" t="n">
-        <v>40</v>
+        <v>264545.4545454545</v>
       </c>
       <c r="K89" t="n">
         <v>0</v>
@@ -22982,7 +22982,7 @@
     </row>
     <row r="90">
       <c r="A90" t="n">
-        <v>70</v>
+        <v>530618.1818181818</v>
       </c>
       <c r="B90" t="inlineStr">
         <is>
@@ -23017,7 +23017,7 @@
         <v>0</v>
       </c>
       <c r="J90" t="n">
-        <v>70</v>
+        <v>530618.1818181818</v>
       </c>
       <c r="K90" t="n">
         <v>0</v>
@@ -23043,7 +23043,7 @@
     </row>
     <row r="91">
       <c r="A91" t="n">
-        <v>40</v>
+        <v>132654.5454545454</v>
       </c>
       <c r="B91" t="inlineStr">
         <is>
@@ -23078,7 +23078,7 @@
         <v>0</v>
       </c>
       <c r="J91" t="n">
-        <v>40</v>
+        <v>132654.5454545454</v>
       </c>
       <c r="K91" t="n">
         <v>0</v>
@@ -23104,7 +23104,7 @@
     </row>
     <row r="92">
       <c r="A92" t="n">
-        <v>44</v>
+        <v>165211.9636363636</v>
       </c>
       <c r="B92" t="inlineStr">
         <is>
@@ -23139,7 +23139,7 @@
         <v>0</v>
       </c>
       <c r="J92" t="n">
-        <v>44</v>
+        <v>165211.9636363636</v>
       </c>
       <c r="K92" t="n">
         <v>0</v>
@@ -23165,7 +23165,7 @@
     </row>
     <row r="93">
       <c r="A93" t="n">
-        <v>32</v>
+        <v>40000</v>
       </c>
       <c r="B93" t="inlineStr">
         <is>
@@ -23203,7 +23203,7 @@
         <v>0</v>
       </c>
       <c r="K93" t="n">
-        <v>16</v>
+        <v>20000</v>
       </c>
       <c r="L93" t="n">
         <v>0</v>
@@ -23221,12 +23221,12 @@
         <v>0</v>
       </c>
       <c r="Q93" t="n">
-        <v>16</v>
+        <v>20000</v>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="n">
-        <v>114</v>
+        <v>0</v>
       </c>
       <c r="B94" t="inlineStr">
         <is>
@@ -23276,18 +23276,18 @@
         <v>0</v>
       </c>
       <c r="O94" t="n">
-        <v>38</v>
+        <v>0</v>
       </c>
       <c r="P94" t="n">
-        <v>38</v>
+        <v>0</v>
       </c>
       <c r="Q94" t="n">
-        <v>38</v>
+        <v>0</v>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="n">
-        <v>64</v>
+        <v>618018.1799999999</v>
       </c>
       <c r="B95" t="inlineStr">
         <is>
@@ -23334,10 +23334,10 @@
         <v>0</v>
       </c>
       <c r="N95" t="n">
-        <v>35</v>
+        <v>309009.09</v>
       </c>
       <c r="O95" t="n">
-        <v>29</v>
+        <v>309009.09</v>
       </c>
       <c r="P95" t="n">
         <v>0</v>
@@ -23348,7 +23348,7 @@
     </row>
     <row r="96">
       <c r="A96" t="n">
-        <v>29</v>
+        <v>3386849.13</v>
       </c>
       <c r="B96" t="inlineStr">
         <is>
@@ -23383,7 +23383,7 @@
         <v>0</v>
       </c>
       <c r="J96" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="K96" t="n">
         <v>0</v>
@@ -23401,7 +23401,7 @@
         <v>0</v>
       </c>
       <c r="P96" t="n">
-        <v>22</v>
+        <v>3386849.13</v>
       </c>
       <c r="Q96" t="n">
         <v>0</v>
@@ -23409,7 +23409,7 @@
     </row>
     <row r="97">
       <c r="A97" t="n">
-        <v>38</v>
+        <v>3683090.92</v>
       </c>
       <c r="B97" t="inlineStr">
         <is>
@@ -23432,7 +23432,7 @@
         </is>
       </c>
       <c r="F97" t="n">
-        <v>5</v>
+        <v>26881.82</v>
       </c>
       <c r="G97" t="n">
         <v>0</v>
@@ -23462,7 +23462,7 @@
         <v>0</v>
       </c>
       <c r="P97" t="n">
-        <v>33</v>
+        <v>3656209.1</v>
       </c>
       <c r="Q97" t="n">
         <v>0</v>
@@ -23470,7 +23470,7 @@
     </row>
     <row r="98">
       <c r="A98" t="n">
-        <v>52</v>
+        <v>2127353.28</v>
       </c>
       <c r="B98" t="inlineStr">
         <is>
@@ -23517,13 +23517,13 @@
         <v>0</v>
       </c>
       <c r="N98" t="n">
-        <v>5</v>
+        <v>709118.4199999999</v>
       </c>
       <c r="O98" t="n">
-        <v>36</v>
+        <v>709117.4299999999</v>
       </c>
       <c r="P98" t="n">
-        <v>11</v>
+        <v>709117.4299999999</v>
       </c>
       <c r="Q98" t="n">
         <v>0</v>
@@ -23531,7 +23531,7 @@
     </row>
     <row r="99">
       <c r="A99" t="n">
-        <v>82</v>
+        <v>2319180.61</v>
       </c>
       <c r="B99" t="inlineStr">
         <is>
@@ -23554,7 +23554,7 @@
         </is>
       </c>
       <c r="F99" t="n">
-        <v>6</v>
+        <v>30053.33</v>
       </c>
       <c r="G99" t="n">
         <v>0</v>
@@ -23569,7 +23569,7 @@
         <v>0</v>
       </c>
       <c r="K99" t="n">
-        <v>6</v>
+        <v>41818.18</v>
       </c>
       <c r="L99" t="n">
         <v>0</v>
@@ -23584,15 +23584,15 @@
         <v>0</v>
       </c>
       <c r="P99" t="n">
-        <v>35</v>
+        <v>1123654.55</v>
       </c>
       <c r="Q99" t="n">
-        <v>35</v>
+        <v>1123654.55</v>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="n">
-        <v>8</v>
+        <v>10000</v>
       </c>
       <c r="B100" t="inlineStr">
         <is>
@@ -23627,7 +23627,7 @@
         <v>0</v>
       </c>
       <c r="J100" t="n">
-        <v>4</v>
+        <v>5000</v>
       </c>
       <c r="K100" t="n">
         <v>0</v>
@@ -23645,7 +23645,7 @@
         <v>0</v>
       </c>
       <c r="P100" t="n">
-        <v>4</v>
+        <v>5000</v>
       </c>
       <c r="Q100" t="n">
         <v>0</v>

</xml_diff>